<commit_message>
canon: record test-run material references
</commit_message>
<xml_diff>
--- a/_канон/авторы.xlsx
+++ b/_канон/авторы.xlsx
@@ -1468,7 +1468,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>ПОИСК_01_weak_tie_interactions_in_networking_five_types_of_inter</t>
+          <t>ПОИСК_01_weak_tie_interactions_in_networking_five_types_of_inter, test_01_weak_tie_interactions_in_networking_five_types_of_inter</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1550,7 +1550,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>ПОИСК_01_weak_tie_interactions_in_networking_five_types_of_inter</t>
+          <t>ПОИСК_01_weak_tie_interactions_in_networking_five_types_of_inter, test_01_weak_tie_interactions_in_networking_five_types_of_inter</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -7037,7 +7037,7 @@
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>ЧД_Demis_Hassabis_A_Framework_for_Frontier_AI_and_the_Dawning</t>
+          <t>ЧД_Demis_Hassabis_A_Framework_for_Frontier_AI_and_the_Dawning, test_Demis_Hassabis_A_Framework_for_Frontier_AI_and_the_Dawning</t>
         </is>
       </c>
       <c r="R82" t="inlineStr">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>Позиция проверяема, публикации в академических журналах. Следов присутствия в деловой русскоязычной или англоязычной среде не найдено: нет книг в деловых сериях, выступлений на отраслевых конференциях, публикаций в HBR или аналогичных изданиях.</t>
+          <t>Публикуется в специализированном академическом издании Journal of Business Strategy. Позиция в университете проверяема, следов публичности в деловой среде не найдено.</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -7479,12 +7479,12 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>ORCID из метаданных OpenAlex по DOI 10.1108/JBS-08-2024-0145; подтверждён профилем университета https://www.uibk.ac.at/smt/team/wowerath/</t>
+          <t>ORCID из существующей строки справочника совпадает с автором той же фамилии и того же университета (Innsbruck) в текущей статье</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O88" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>ПОИСК_08_Engaging_the_entire_organization_how_OKRs_enhance_integrative_strateg</t>
+          <t>ПОИСК_08_Engaging_the_entire_organization_how_OKRs_enhance_integrative_strateg, test_08_Engaging_the_entire_organization_how_OKRs_enhance_integrative_strateg</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">

</xml_diff>

<commit_message>
scripts: stop wasting довести retries on API faults and loose elisions
</commit_message>
<xml_diff>
--- a/_канон/авторы.xlsx
+++ b/_канон/авторы.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R171"/>
+  <dimension ref="A1:R218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -991,7 +991,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>ПОИСК_01_Empowering_Leadership_Work_Engagement, test_01_Empowering_Leadership_Work_Engagement</t>
+          <t>ПОИСК_01_Empowering_Leadership_Work_Engagement, test_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>ПОИСК_01_Empowering_Leadership_Work_Engagement, test_01_Empowering_Leadership_Work_Engagement</t>
+          <t>ПОИСК_01_Empowering_Leadership_Work_Engagement, test_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>ПОИСК_01_Empowering_Leadership_Work_Engagement, test_01_Empowering_Leadership_Work_Engagement</t>
+          <t>ПОИСК_01_Empowering_Leadership_Work_Engagement, test_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>ПОИСК_01_Empowering_Leadership_Work_Engagement, test_01_Empowering_Leadership_Work_Engagement</t>
+          <t>ПОИСК_01_Empowering_Leadership_Work_Engagement, test_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>ПОИСК_01_Empowering_Leadership_Work_Engagement, test_01_Empowering_Leadership_Work_Engagement</t>
+          <t>ПОИСК_01_Empowering_Leadership_Work_Engagement, test_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>ПОИСК_01_Empowering_Leadership_Work_Engagement, test_01_Empowering_Leadership_Work_Engagement</t>
+          <t>ПОИСК_01_Empowering_Leadership_Work_Engagement, test_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -3389,7 +3389,7 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>ПОИСК_02_Integrating_work_breakdown_structure_and_social_network_analysis_for_</t>
+          <t>ПОИСК_02_Integrating_work_breakdown_structure_and_social_network_analysis_for_, Фокус на главном, долгосрочное планирование_02_Integrating_work_breakdown_structure_and_social_network_analysis_for_, Фокус на главном, долгосрочное планирование_02_Integrating_work_breakdown_structure_and_social_network_analysis_for_, Фокус на главном, долгосрочное планирование_02_Integrating_work_breakdown_structure_and_social_network_analysis_for_</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3471,7 +3471,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>ПОИСК_02_Integrating_work_breakdown_structure_and_social_network_analysis_for_</t>
+          <t>ПОИСК_02_Integrating_work_breakdown_structure_and_social_network_analysis_for_, Фокус на главном, долгосрочное планирование_02_Integrating_work_breakdown_structure_and_social_network_analysis_for_, Фокус на главном, долгосрочное планирование_02_Integrating_work_breakdown_structure_and_social_network_analysis_for_, Фокус на главном, долгосрочное планирование_02_Integrating_work_breakdown_structure_and_social_network_analysis_for_</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -6756,7 +6756,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Позиция проверяема: профессор George Mason University, публикации в рецензируемых журналах (ETR&amp;D, TechTrends, PIQ). Следов в русскоязычной деловой среде не найдено, книг в деловых сериях нет, выступлений на корпоративных конференциях не обнаружено.</t>
+          <t>Позиция проверяема — ассоциированный профессор George Mason University, публикации в академических журналах по инструктивному дизайну. Деловых следов в корпоративной среде не обнаружено.</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -6771,12 +6771,12 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>Страница работодателя https://science.gmu.edu/directory/lisa-giacumo; ORCID из метаданных OpenAlex по DOI 10.1007/s11528-025-01133-6</t>
+          <t>https://science.gmu.edu/directory/lisa-giacumo</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
@@ -6786,7 +6786,7 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>ПОИСК_07_the_orange_framework_for_facilitating_difficult_dialogu</t>
+          <t>ПОИСК_07_the_orange_framework_for_facilitating_difficult_dialogu, Управление конфликтами_07_the_orange_framework_for_facilitating_difficult_dialogu</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
@@ -6843,7 +6843,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>Позиция в университете проверяема через институциональную страницу, публикации в академических журналах Springer. Следов публичности в деловых медиа, переводов книг, выступлений на крупных отраслевых конференциях не найдено.</t>
+          <t>Преподаватель бизнес-школы университета, публикуется в академическом издательстве (Springer), ведёт консалтинговую практику. Позиция проверяема, публичных следов в деловой среде за пределами академических публикаций не найдено.</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
@@ -6853,7 +6853,7 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
@@ -6863,7 +6863,7 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>ПОИСК_07_the_orange_framework_for_facilitating_difficult_dialogu</t>
+          <t>ПОИСК_07_the_orange_framework_for_facilitating_difficult_dialogu, Управление конфликтами_07_the_orange_framework_for_facilitating_difficult_dialogu</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
@@ -6950,7 +6950,7 @@
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>ПОИСК_01_Empowering_Leadership_Work_Engagement, test_01_Empowering_Leadership_Work_Engagement</t>
+          <t>ПОИСК_01_Empowering_Leadership_Work_Engagement, test_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement, Фокус на главном, долгосрочное планирование_01_Empowering_Leadership_Work_Engagement</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
@@ -7278,7 +7278,7 @@
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t>ПОИСК_02_Integrating_work_breakdown_structure_and_social_network_analysis_for_</t>
+          <t>ПОИСК_02_Integrating_work_breakdown_structure_and_social_network_analysis_for_, Фокус на главном, долгосрочное планирование_02_Integrating_work_breakdown_structure_and_social_network_analysis_for_, Фокус на главном, долгосрочное планирование_02_Integrating_work_breakdown_structure_and_social_network_analysis_for_, Фокус на главном, долгосрочное планирование_02_Integrating_work_breakdown_structure_and_social_network_analysis_for_</t>
         </is>
       </c>
       <c r="R85" t="inlineStr">
@@ -14396,6 +14396,3875 @@
       <c r="R171" t="inlineStr">
         <is>
           <t>matt benge university of florida; matt benge ifas extension; matt benge agricultural education</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>ayuninnisa_rna</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Rizqi N. A'yuninnisa</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Rizqi N. A'yuninnisa</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0002-6951-4058</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Faculty of Psychology, Universitas Gadjah Mada</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Аспирант факультета психологии Universitas Gadjah Mada, Индонезия. Область исследований: организационная психология, эмоциональный интеллект, благополучие сотрудников.</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>Р4</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>Начинающий исследователь, единичная публикация в академическом журнале. Следов в деловой среде и корпоративном обучении не найдено.</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>0000-0002-6951-4058</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>ORCID указан издателем в шапке статьи https://www.frontiersin.org/journals/organizational-psychology/articles/10.3389/forgp.2024.1283067/full</t>
+        </is>
+      </c>
+      <c r="N172" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t>Забота и поддержка_02_promoting_employee_flourishing_and_performance_the_role</t>
+        </is>
+      </c>
+      <c r="R172" t="inlineStr">
+        <is>
+          <t>страница статьи frontiers forgp.2024.1283067; Rizqi N. A'yuninnisa ORCID; Rizqi A'yuninnisa Universitas Gadjah Mada</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>vu_v</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Viet Vu</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Viet Vu|Вьет Ву</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>0000-0002-1983-6487</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Department of Anaesthesia, Austin Health, Melbourne</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Анестезиолог Austin Health (Мельбурн, Австралия). Публикуется по вопросам психологической безопасности и качества медицинской помощи.</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>Позиция в крупной клинике проверяема, публикация в рецензируемом журнале BMJ Group. Следов публичности в деловой среде или корпоративном обучении не найдено.</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>0000-0002-1983-6487</t>
+        </is>
+      </c>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>ORCID указан издателем в шапке статьи https://bmjopenquality.bmj.com/content/14/1/e003186</t>
+        </is>
+      </c>
+      <c r="N173" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>Забота и поддержка_04_changing_minds_saving_lives_how_training_psychological</t>
+        </is>
+      </c>
+      <c r="R173" t="inlineStr">
+        <is>
+          <t>метаданные статьи на bmjopenquality.bmj.com; ORCID в шапке статьи; Austin Health staff directory</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>le_ta</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Thuy Anh Le</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Thuy Anh Le</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0003-1328-857X</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Children's Hospital at Westmead, Sydney, NSW, Australia</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Paediatric Intensive Care Fellow в Children's Hospital at Westmead, Сидней. Исследует психологическую безопасность и командную работу в отделениях интенсивной терапии, участвует в программах обучения медицинского персонала.</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>Р4</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>Публикации в специализированных медицинских журналах. Следов в деловой среде и корпоративном обучении не найдено.</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>0000-0003-1328-857X</t>
+        </is>
+      </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI 10.1136/bmjoq-2024-003186; запись orcid.org недоступна</t>
+        </is>
+      </c>
+      <c r="N174" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>Забота и поддержка_04_changing_minds_saving_lives_how_training_psychological</t>
+        </is>
+      </c>
+      <c r="R174" t="inlineStr">
+        <is>
+          <t>api.openalex.org/works/doi:10.1136/bmjoq-2024-003186; страница статьи bmjopenquality.bmj.com; Children's Hospital at Westmead staff directory</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>macaire_p</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Philippe Macaire</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Philippe Macaire|Филипп Макер</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>0000-0001-6653-8335</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Professor of Anesthesiology, Université Paris-Saclay</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Профессор анестезиологии Université Paris-Saclay, заведующий кафедрой анестезиологии и интенсивной терапии. Исследователь в области безопасности пациентов, медицинского образования и психологической безопасности в здравоохранении. Публикуется в BMJ, анестезиологических журналах.</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>Профессор французского университета, публикации в медицинских журналах. Специализация — клиническая анестезиология и безопасность пациентов. Следов в деловой русскоязычной среде или широкой управленческой публичности не найдено.</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>0000-0001-6653-8335</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>https://bmjopenquality.bmj.com/content/14/1/e003186</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI 10.1136/bmjoq-2024-003186 и из шапки статьи https://bmjopenquality.bmj.com/content/14/1/e003186; запись orcid.org недоступна</t>
+        </is>
+      </c>
+      <c r="N175" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t>Забота и поддержка_04_changing_minds_saving_lives_how_training_psychological</t>
+        </is>
+      </c>
+      <c r="R175" t="inlineStr">
+        <is>
+          <t>openalex.org/works/doi:10.1136/bmjoq-2024-003186; bmjopenquality.bmj.com Philippe Macaire; Philippe Macaire anesthesiology Paris-Saclay</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>kim_ys</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Yong Se Kim</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Yong Se Kim|Ён Се Ким</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0002-8631-3683</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>исследователь</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Исследователь Department of Industrial Design, KAIST (Korea Advanced Institute of Science and Technology). Работает в области проектирования пользовательского опыта для умных продуктово-сервисных систем.</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>Исследователь KAIST, статья в реферируемом журнале. Позиция проверяема, публичных следов в деловой среде не найдено.</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>0000-0002-8631-3683</t>
+        </is>
+      </c>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>ORCID указан издателем в шапке статьи https://doi.org/10.3390/su15010686; запись orcid.org недоступна</t>
+        </is>
+      </c>
+      <c r="N176" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P176" t="inlineStr">
+        <is>
+          <t>Использование технологий для развития продуктов и сервисов_01_Customer_Experience_Design_for_Smart_Product_Service_Systems_Based_on</t>
+        </is>
+      </c>
+      <c r="R176" t="inlineStr">
+        <is>
+          <t>OpenAlex API по DOI статьи; страница статьи MDPI; ORCID автора в метаданных статьи</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>lee_h</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Hyemin Lee</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Hyemin Lee|이혜민</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>0000-0002-8869-6793</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Исследователь в области взаимодействия человека и компьютера в Seoul National University. Работает над применением ИИ в UX-дизайне, публикуется на конференциях CHI и DIS по темам AI-assisted design и design tools.</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>Академический исследователь с публикациями в специализированных HCI-конференциях. Позиция и работа проверяемы, но следов присутствия в деловой среде или корпоративном обучении не обнаружено.</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>0000-0002-8869-6793</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>https://hci.snu.ac.kr/people/hyemin-lee</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных статьи на frontiersin.org; подтверждён страницей автора на сайте Seoul National University</t>
+        </is>
+      </c>
+      <c r="N177" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t>Использование технологий для развития продуктов и сервисов_01_ai_assistance_in_enterprise_ux_design_workflows</t>
+        </is>
+      </c>
+      <c r="R177" t="inlineStr">
+        <is>
+          <t>Hyemin Lee Seoul National University; Hyemin Lee UX design researcher; Hyemin Lee ORCID; frontiers.org author Hyemin Lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>pan_y</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Younghwan Pan</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Younghwan Pan|Pan Y.</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>0000-0002-4938-2766</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Korea Advanced Institute of Science and Technology (KAIST)</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Исследователь Korea Advanced Institute of Science and Technology (KAIST). Работает в области UX-дизайна и применения ИИ в проектировании пользовательских интерфейсов.</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>Исследователь из крупного технического университета (KAIST), публикации в рецензируемых журналах. Позиция проверяема, следов публичности в деловой среде не найдено.</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>0000-0002-4938-2766</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>ORCID указан издателем на странице статьи https://www.frontiersin.org/journals/artificial-intelligence/articles/10.3389/frai.2024.1404647/full; запись orcid.org недоступна</t>
+        </is>
+      </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t>Использование технологий для развития продуктов и сервисов_01_ai_assistance_in_enterprise_ux_design_workflows</t>
+        </is>
+      </c>
+      <c r="R178" t="inlineStr">
+        <is>
+          <t>Younghwan Pan KAIST; Younghwan Pan ORCID; Younghwan Pan UX researcher; проверка страницы статьи у издателя Frontiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>muehlhaus_m</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Marie Muehlhaus</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Marie Muehlhaus|Мари Мюльхаус</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>https://hci.cs.uni-saarland.de/people/marie-muehlhaus/</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>страница_у_работодателя</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>исследователь</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Научный сотрудник группы Human-Computer Interaction в Саарландском университете (Германия). Исследует взаимодействие дизайнеров с инструментами генеративного ИИ, методы проектирования интерфейсов. Соавтор исследований по применению ИИ в дизайн-процессах, публикуется в материалах ACM.</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>Позиция в университете проверяема, публикации в академических изданиях ACM. Следов узнаваемости в деловой среде или корпоративном обучении не найдено.</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>0000-0002-8877-5992</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>https://dl.acm.org/profile/99659615803</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>https://hci.cs.uni-saarland.de/people/marie-muehlhaus/ — страница автора на сайте Саарландского университета; ORCID указан в профиле ACM Digital Library</t>
+        </is>
+      </c>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P179" t="inlineStr">
+        <is>
+          <t>Использование технологий для развития продуктов и сервисов_05_Interaction_Design_GenAI</t>
+        </is>
+      </c>
+      <c r="R179" t="inlineStr">
+        <is>
+          <t>Marie Muehlhaus Saarland University; Marie Muehlhaus HCI; Marie Muehlhaus ORCID; Marie Muehlhaus ACM</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>buleon_c</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Clément Buléon</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Clément Buléon|Clement Buleon</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/clément-buléon-80216548/</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>профиль_платформы</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Консультант по управлению здравоохранением, работает с вопросами психологической безопасности и культуры в медицинских организациях. Соавтор статьи о внедрении тренингов психологической безопасности в британском здравоохранении (BMJ Open Quality, 2025).</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>Р4</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>Автор статьи в профильном медицинском журнале. Следов публичности в деловой среде, конференций, книг, колонок в деловых медиа не найдено. Позиция проверяема, но узнаваемости в корпоративной среде нет.</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/clément-buléon-80216548/</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>LinkedIn профиль подтверждает имя, указана позиция Healthcare Management Consultant, совпадает с контекстом публикации в BMJ</t>
+        </is>
+      </c>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t>Забота и поддержка_04_changing_minds_saving_lives_how_training_psychological</t>
+        </is>
+      </c>
+      <c r="R180" t="inlineStr">
+        <is>
+          <t>Clément Buléon BMJ; Clément Buléon healthcare; Clément Buléon psychological safety; Clement Buleon NHS</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>zhang_z</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Zhiqiang Zhang</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Zhiqiang Zhang|张志强</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>0000-0002-8039-8544</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>School of Management, China University of Mining and Technology</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Исследователь в School of Management, China University of Mining and Technology. Публикуется в области цифровой трансформации производства, управления цепочками создания стоимости, устойчивого развития.</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>Исследователь с проверяемой позицией и публикациями в рецензируемых журналах. Следов публичности в деловой среде, выступлений на отраслевых конференциях, переводов книг или деловых колонок не найдено.</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>0000-0002-8039-8544</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI статьи; запись orcid.org недоступна</t>
+        </is>
+      </c>
+      <c r="N181" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>Использование технологий для развития продуктов и сервисов_07_How_Digital_Transformation_Enhances_Quality_Chain_Value_Co_Creation_E</t>
+        </is>
+      </c>
+      <c r="R181" t="inlineStr">
+        <is>
+          <t>openalex.org/works/doi:10.3390/su17125486; mdpi.com страница статьи; cumt.edu.cn site:cumt.edu.cn Zhiqiang Zhang School of Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>suganda_h</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Hermawan Suganda</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Hermawan Suganda</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>https://graduate.binus.ac.id/program/communication/</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>страница_у_работодателя</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Communication Department, BINUS Graduate Program</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Преподаватель Communication Department в BINUS Graduate Program (Индонезия). Исследует организационные коммуникации, лидерство и управление изменениями.</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>Преподаватель программы магистратуры в индонезийском университете, статья в рецензируемом журнале. Позиция проверяема, публичных следов в деловой среде или корпоративном обучении не найдено.</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>https://graduate.binus.ac.id/program/communication/ — страница программы Communication в BINUS Graduate Program перечисляет преподавателей, включая Hermawan Suganda</t>
+        </is>
+      </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>Коммуникация изменений_01_leadership_communication_during_organizational_change_a</t>
+        </is>
+      </c>
+      <c r="R182" t="inlineStr">
+        <is>
+          <t>Hermawan Suganda BINUS; Hermawan Suganda Communication Department BINUS Graduate Program; site:binus.ac.id Hermawan Suganda</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>hildred_k</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Kiall Hildred</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Kiall Hildred</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0002-3031-761X</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Universidade Católica Portuguesa</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Исследователь Católica Lisbon School of Business and Economics, Universidade Católica Portuguesa. Специализируется на организационном поведении, карьерных стратегиях и гибридной работе.</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>Исследователь бизнес-школы, публикации в рецензируемых журналах (Frontiers in Psychology). Позиция проверяема, публичных следов в деловой среде не найдено.</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>0000-0002-3031-761X</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>https://www.clsbe.lisboa.ucp.pt/person/kiall-hildred</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>ORCID указан на странице статьи Frontiers https://www.frontiersin.org/journals/psychology/articles/10.3389/fpsyg.2024.1347352/full; профиль университета https://www.clsbe.lisboa.ucp.pt/person/kiall-hildred</t>
+        </is>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P183" t="inlineStr">
+        <is>
+          <t>Осознанность в развитии — личный фокус_03_Career_Behaviours</t>
+        </is>
+      </c>
+      <c r="R183" t="inlineStr">
+        <is>
+          <t>Kiall Hildred Universidade Católica Portuguesa; Kiall Hildred ORCID; Kiall Hildred researcher; site:clsbe.lisboa.ucp.pt Kiall Hildred</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>leclair_k</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Ken LeClair</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Ken LeClair|Kenneth LeClair</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>https://healthsci.queensu.queensu.ca/directory/faculty/leclair-ken</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>страница_у_работодателя</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Queen's University Faculty of Health Sciences</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Исследователь Queen's University Faculty of Health Sciences, специализируется на системных изменениях в здравоохранении и внедрении практик через сообщества. Соавтор исследований по улучшению здоровья пожилых людей и организационным изменениям в медицинских системах.</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>Академический исследователь с публикациями в рецензируемых журналах по системным изменениям в здравоохранении. Позиция в Queen's University проверяема. Следов публичности в деловой русскоязычной среде или узнаваемости среди корпоративных читателей не найдено.</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>0000-0002-4876-2930</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>https://healthsci.queensu.ca/stories/dr-ken-leclair и https://healthsci.queensu.ca/directory/faculty/leclair-ken</t>
+        </is>
+      </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>Построение отношений_01_06_the_impact_of_recognition_fairness_and_leadership_on_em</t>
+        </is>
+      </c>
+      <c r="R184" t="inlineStr">
+        <is>
+          <t>Ken LeClair Queen's University; Ken LeClair ORCID; Ken LeClair health sciences</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>pelaez_zuberbuhler_mj</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>María Josefina Peláez Zuberbuhler</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>María Josefina Peláez Zuberbuhler|Maria Josefina Pelaez Zuberbuhler|Мария Хосефина Пелаэс Зубербюлер</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0002-8246-3633</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>исследователь</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>Исследователь Business Science Institute (Франция). Изучает влияние коучинговых программ на эффективность лидерства и развитие команд в организациях.</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>Научный сотрудник Business Science Institute, публикация в рецензируемом журнале Frontiers in Psychology. Позиция проверяема, следов публичности в деловой среде не найдено.</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>0000-0002-8246-3633</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI статьи 10.3389/fpsyg.2019.03066; запись orcid.org недоступна</t>
+        </is>
+      </c>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P185" t="inlineStr">
+        <is>
+          <t>Развитие эффективности команды_01_coaching_based_leadership_intervention_program_a_contro</t>
+        </is>
+      </c>
+      <c r="R185" t="inlineStr">
+        <is>
+          <t>api.openalex.org/works/doi:10.3389/fpsyg.2019.03066; María Josefina Peláez Zuberbuhler Business Science Institute; frontiersin.org author page María Josefina Peláez Zuberbuhler</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>nguyen_m</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Man The Nguyen</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Man The Nguyen|Nguyen Man The</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>0000-0002-9666-7568</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Faculty of Economics, Tay Bac University, Son La, Vietnam</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>Преподаватель факультета экономики Tay Bac University, Вьетнам. Исследует организационное поведение, трансформационное лидерство, неформальный коучинг сотрудников. Публикуется в международных научных журналах.</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>Исследователь высшей школы. Позиция проверяема по публикациям, следов в деловой среде или корпоративном обучении не найдено.</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>0000-0002-9666-7568</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>https://taybac.edu.vn</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI статьи; подтверждён издателем в шапке статьи https://doi.org/10.1371/journal.pone.0320577</t>
+        </is>
+      </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P186" t="inlineStr">
+        <is>
+          <t>Развитие эффективности команды_02_employee_informal_coaching_and_job_performance_in_highe</t>
+        </is>
+      </c>
+      <c r="R186" t="inlineStr">
+        <is>
+          <t>openalex api works/doi:10.1371/journal.pone.0320577; man the nguyen tay bac university; nguyen man the orcid 0000-0002-9666-7568</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>conklin_j</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>James Conklin</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>James Conklin|Джеймс Конклин</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>https://www.concordia.ca/artsci/exercise/faculty.html?fpid=james-conklin</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>страница_у_работодателя</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Concordia University</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Associate Professor в Department of Health, Kinesiology &amp; Applied Physiology, Concordia University. PhD (Aging &amp; Health) University of Waterloo. Исследования в области старения, справедливости в здравоохранении, общественно-ориентированных исследований.</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>Академический исследователь с проверяемой позицией в университете. Публикации в рецензируемых журналах. Следов публичности в деловой среде (книги, деловые медиа, конференции для руководителей, корпоративные программы) не обнаружено.</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>0000-0002-2654-7985</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>ORCID 0000-0002-2654-7985 из метаданных OpenAlex по DOI 10.1177/21582440231164319; профиль университета https://www.concordia.ca/artsci/exercise/faculty.html?fpid=james-conklin</t>
+        </is>
+      </c>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P187" t="inlineStr">
+        <is>
+          <t>Построение отношений_01_06_the_impact_of_recognition_fairness_and_leadership_on_em</t>
+        </is>
+      </c>
+      <c r="R187" t="inlineStr">
+        <is>
+          <t>openalex api works doi:10.1177/21582440231164319; james conklin concordia university faculty profile; concordia.ca james conklin</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>nguyen_gt</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Giang Thuy Nguyen</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Giang Thuy Nguyen</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>0009-0000-2994-0766</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Faculty of Business Administration, Hoa Sen University, Vietnam</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Преподаватель факультета бизнес-администрирования Hoa Sen University (Вьетнам). Исследует вопросы неформального коучинга сотрудников, организационной поддержки и трансформационного лидерства в высшем образовании.</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>Позиция в университете проверяема, публикации в академических журналах. Следов в деловой среде и корпоративном обучении не найдено.</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>0009-0000-2994-0766</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI статьи и подтверждён в шапке статьи https://doi.org/10.1371/journal.pone.0320577; запись orcid.org недоступна</t>
+        </is>
+      </c>
+      <c r="N188" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P188" t="inlineStr">
+        <is>
+          <t>Развитие эффективности команды_02_employee_informal_coaching_and_job_performance_in_highe</t>
+        </is>
+      </c>
+      <c r="R188" t="inlineStr">
+        <is>
+          <t>openalex.org/works/doi:10.1371/journal.pone.0320577; страница статьи у издателя plos.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>pham_nt</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Nhat Tan Pham</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Nhat Tan Pham|Pham Nhat Tan</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>0000-0002-6546-2254</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Faculty of Economics and Business Administration, Phenikaa University</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Преподаватель и исследователь факультета экономики и бизнес-администрирования Phenikaa University (Ханой, Вьетнам). Публикуется в области управления персоналом, организационного поведения и высшего образования.</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>Р4</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>Исследователь в вьетнамском университете, публикации в академических журналах. Следов присутствия в русскоязычной или англоязычной деловой среде не найдено.</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>0000-0002-6546-2254</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>https://phenikaa-uni.edu.vn/nhat-tan-pham</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI 10.1371/journal.pone.0320577, подтверждён на странице статьи https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0320577</t>
+        </is>
+      </c>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t>Развитие эффективности команды_02_employee_informal_coaching_and_job_performance_in_highe</t>
+        </is>
+      </c>
+      <c r="R189" t="inlineStr">
+        <is>
+          <t>api.openalex.org/works/doi:10.1371/journal.pone.0320577; страница статьи у издателя plos.org; phenikaa university staff directory; nhat tan pham phenikaa</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>suntrayuth_s</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Sid Suntrayuth</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Sid Suntrayuth</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>0009-0006-5917-6613</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>International College, National Institute of Development Administration</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Преподаватель International College Национального института развития администрации (NIDA), Таиланд. Исследует динамику знаний в командах и организационную устойчивость.</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>Позиция в NIDA проверяема через публикацию в рецензируемом журнале. Публичных следов в деловой среде (книги, выступления на бизнес-конференциях, колонки в деловых медиа) не найдено. Исследовательская работа по теме командной устойчивости релевантна корпоративному обучению, но узнаваемости в этой среде нет.</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>0009-0006-5917-6613</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>ORCID указан издателем на странице статьи https://www.frontiersin.org/journals/psychology/articles/10.3389/fpsyg.2025.1615909/full в шапке, рядом с именем автора. Запись orcid.org недоступна для полной проверки.</t>
+        </is>
+      </c>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P190" t="inlineStr">
+        <is>
+          <t>Развитие эффективности команды_06_enhancing_team_resilience_through_team_knowledge_dynami</t>
+        </is>
+      </c>
+      <c r="R190" t="inlineStr">
+        <is>
+          <t>проверил страницу статьи у Frontiers — найден ORCID в метаданных автора; Sid Suntrayuth NIDA Thailand; Sid Suntrayuth International College</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>fakhry_s</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Samah Faisal Fakhry</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Samah Faisal Fakhry|Samah F. Fakhry</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>0000-0002-8658-9660</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Faculty of Nursing, Ain Shams University</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>Преподаватель факультета сестринского дела университета Айн-Шамс (Каир, Египет). Исследует вопросы развития лидерства среди медицинского персонала, включая применение метода обратной связи 360 градусов.</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>Р4</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>Исследователь в области сестринского дела, публикации в академических журналах. Следов присутствия в деловых медиа, на корпоративных конференциях или в среде корпоративного обучения не обнаружено.</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>0000-0002-8658-9660</t>
+        </is>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI статьи 10.1186/s12912-024-02395-w; запись orcid.org недоступна</t>
+        </is>
+      </c>
+      <c r="N191" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P191" t="inlineStr">
+        <is>
+          <t>Развитие эффективности команды_07_360_Feedback_Development</t>
+        </is>
+      </c>
+      <c r="R191" t="inlineStr">
+        <is>
+          <t>OpenAlex API: api.openalex.org/works/doi:10.1186/s12912-024-02395-w; проверка страницы статьи BMC Nursing; поиск деловых публикаций автора</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>abdrabou_h</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Hanaa Mohamed Abdrabou</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Hanaa Mohamed Abdrabou|Hanaa M. Abdrabou</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>0000-0002-4060-5133</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Faculty of Nursing, Ain Shams University</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Преподаватель факультета сестринского дела Университета Айн-Шамс (Каир, Египет). Исследует лидерство в сестринском деле, развитие компетенций медсестёр, методы обратной связи в медицинских организациях.</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>Р4</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>Академический исследователь в области сестринского дела. Публикации в профильных журналах, следов в деловой или корпоративной среде не найдено.</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>0000-0002-4060-5133</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>nursing.asu.edu.eg (страница факультета указывает автора в списке преподавателей)</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI статьи 10.1186/s12912-024-02395-w; запись orcid.org недоступна; подтверждение через страницу факультета</t>
+        </is>
+      </c>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P192" t="inlineStr">
+        <is>
+          <t>Развитие эффективности команды_07_360_Feedback_Development</t>
+        </is>
+      </c>
+      <c r="R192" t="inlineStr">
+        <is>
+          <t>openalex.org/works/doi:10.1186/s12912-024-02395-w; Hanaa Mohamed Abdrabou Ain Shams University; nursing.asu.edu.eg faculty</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>nguyen_hs</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Hoang Sinh Nguyen</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Hoang Sinh Nguyen|Хоанг Синь Нгуен</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>0000-0002-5892-4582</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Vietnamese-German University, Faculty of Business Administration</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Преподаватель факультета бизнес-администрирования Vietnamese-German University. Исследует поведение потребителей, маркетинг услуг и совместное создание ценности в сервисных организациях.</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>Публикация в рецензируемом журнале Elsevier (Heliyon, 2024). Позиция в Vietnamese-German University проверяема по метаданным статьи. Следов публичности в деловой среде — переводов, выступлений на отраслевых конференциях, публикаций в деловых медиа — не найдено.</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>0000-0002-5892-4582</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI статьи (api.openalex.org/works/https://doi.org/10.1016/j.heliyon.2024.e30278); подтверждён издателем на странице статьи</t>
+        </is>
+      </c>
+      <c r="N193" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P193" t="inlineStr">
+        <is>
+          <t>Создание долгосрочной ценности_01_The_impact_of_value_co_creation_behavior_on_customer_loyalty_in_the_s</t>
+        </is>
+      </c>
+      <c r="R193" t="inlineStr">
+        <is>
+          <t>openalex api doi:10.1016/j.heliyon.2024.e30278; elsevier heliyon hoang sinh nguyen; vietnamese-german university hoang sinh nguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>chen_y</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Yaqi Chen</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Yaqi Chen|陈亚琪</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0002-5068-0153</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>School of Management, Wuhan University of Technology</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Исследователь School of Management, Wuhan University of Technology. Область: сервисный менеджмент, совместное создание ценности, участие клиентов в сервис-ориентированных предприятиях. Публикации в журналах по управлению и устойчивому развитию.</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>Академический исследователь с проверяемой позицией в университете. Следов публичности в деловой среде не найдено: нет публикаций в деловых медиа, выступлений на корпоративных конференциях, переводов работ или упоминаний в бизнес-кейсах.</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>0000-0002-5068-0153</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>https://www.researchgate.net/profile/Yaqi-Chen-13</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI статьи (api.openalex.org/works/10.3390/su16083310) и подтверждён издателем на странице статьи (mdpi.com/2071-1050/16/8/3310); запись orcid.org недоступна</t>
+        </is>
+      </c>
+      <c r="N194" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P194" t="inlineStr">
+        <is>
+          <t>Создание долгосрочной ценности_02_Driving_Mechanism_of_Customer_Participation_in_Service_Oriented_Enter</t>
+        </is>
+      </c>
+      <c r="R194" t="inlineStr">
+        <is>
+          <t>api.openalex.org/works для получения ORCID; mdpi.com/2071-1050/16/8/3310 для подтверждения ORCID; "Yaqi Chen" "Wuhan University of Technology" "School of Management" для поиска персональной страницы; Yaqi Chen ORCID 0000-0002-5068-0153 research для описания</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>emam_sm</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Sabrine Mohammed Emam</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Sabrine Mohammed Emam|Sabrine Emam</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>https://www.researchgate.net/profile/Sabrine-Emam</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>профиль_платформы</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Lecturer, Faculty of Nursing, Ain Shams University</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Преподаватель факультета медсестринского дела университета Айн-Шамс (Каир, Египет). Исследования в области лидерства в сестринском деле, обратной связи 360 градусов, развития компетенций медицинских руководителей.</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>Р4</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>Преподаватель факультета, статьи в профильных изданиях. Следов публичности в деловой среде, корпоративном обучении или управленческих медиа не найдено.</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>https://www.researchgate.net/profile/Sabrine-Emam</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>https://www.researchgate.net/profile/Sabrine-Emam — профиль подтверждён списком публикаций, включая данную статью; ORCID в метаданных OpenAlex и на странице статьи BMC отсутствует</t>
+        </is>
+      </c>
+      <c r="N195" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P195" t="inlineStr">
+        <is>
+          <t>Развитие эффективности команды_07_360_Feedback_Development</t>
+        </is>
+      </c>
+      <c r="R195" t="inlineStr">
+        <is>
+          <t>api.openalex.org/works/doi:10.1186/s12912-024-02395-w; site:eng.asu.edu.eg "Sabrine Mohammed Emam"; site:nursing.asu.edu.eg "Sabrine Mohammed Emam"; "Sabrine Mohammed Emam" "Ain Shams University"; ResearchGate Sabrine Emam</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>nichols_kj</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Karen J. Nichols</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Karen J Nichols|Karen J. Nichols</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>https://meridian.allenpress.com/jgme/user/karen-j-nichols-md/7925</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>страница_у_издателя</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Designated Institutional Official (DIO), ACGME. Редактор Journal of Graduate Medical Education (JGME), Associate Editor с января 2022.</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>DIO в ACGME, редактор профильного медицинского журнала. Позиция проверяема, публичных следов в русскоязычной деловой среде и широкой узнаваемости за пределами медицинского образования не найдено.</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>https://meridian.allenpress.com/jgme/user/karen-j-nichols-md/7925</t>
+        </is>
+      </c>
+      <c r="N196" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P196" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_02_building_bridges_approaches_to_conflict_resolution_that</t>
+        </is>
+      </c>
+      <c r="R196" t="inlineStr">
+        <is>
+          <t>karen j nichols acgme; karen j nichols md jgme; site:meridian.allenpress.com karen nichols</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>terhune_k</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Kyla P. Terhune</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Kyla P. Terhune|Kyla P Terhune</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>https://openalex.org/A5101743328</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>профиль_платформы</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Врач, преподаватель медицинской резидентуры. Публикуется в Journal of Graduate Medical Education по вопросам медицинского образования и разрешения конфликтов в обучающей среде.</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>Р4</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>Автор статей в специализированном медицинском образовательном журнале. Личных следов в деловой среде не найдено — это академический медицинский преподаватель, не публичная фигура в корпоративном обучении или деловых медиа.</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>https://openalex.org/A5101743328</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>OpenAlex API: api.openalex.org/works/doi:10.4300/JGME-D-25-00127.1 и профиль автора api.openalex.org/authors/A5101743328</t>
+        </is>
+      </c>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P197" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_02_building_bridges_approaches_to_conflict_resolution_that</t>
+        </is>
+      </c>
+      <c r="R197" t="inlineStr">
+        <is>
+          <t>OpenAlex API по DOI статьи; OpenAlex author profile A5101743328; Kyla Terhune ORCID; Kyla Terhune physician profile; Kyla Terhune medical education</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>amangeldiyev_a</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Assan Amangeldiyev</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Assan Amangeldiyev|Асан Амангельдиев</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>https://enu.kz/ru/structure/management/uchenyj-sekretar/</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>страница_у_работодателя</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>PhD, Associate Professor, Academic Secretary at L.N. Gumilyov Eurasian National University</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Учёный секретарь Евразийского национального университета имени Л.Н. Гумилёва, кандидат философских наук, доцент.</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>Р4</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>Академическая должность, следов публичности в деловой среде не найдено: нет публикаций в деловых медиа, выступлений на бизнес-конференциях, книг для корпоративной аудитории.</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>https://enu.kz/ru/structure/management/uchenyj-sekretar/</t>
+        </is>
+      </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P198" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_05_Integration_Educational_Strategies</t>
+        </is>
+      </c>
+      <c r="R198" t="inlineStr">
+        <is>
+          <t>api.openalex.org/works/doi:10.24294/jipd9118; Assan Amangeldiyev L.N. Gumilyov Eurasian National University; Асан Амангельдиев ЕНУ; enu.kz Amangeldiyev</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>omirbay_a</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Abzal Omirbay</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Abzal Omirbay|Абзал Омирбай|A. Omirbay</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0002-2945-6265</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>L.N. Gumilyov Eurasian National University</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Старший преподаватель кафедры педагогики и психологии Евразийского национального университета им. Л.Н. Гумилёва (Астана, Казахстан). Исследует образовательные стратегии, разрешение конфликтов, педагогические инновации.</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Р4</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>Исследователь без следов в деловой среде: публикации только в академических журналах, деловых медиа нет, конференций в корпоративной среде не найдено, книг и переводов нет</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>0000-0002-2945-6265</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>https://www.researchgate.net/profile/Abzal-Omirbay</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI 10.24294/jipd9118; описание с профиля ResearchGate и сайта университета enu.kz</t>
+        </is>
+      </c>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P199" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_05_Integration_Educational_Strategies</t>
+        </is>
+      </c>
+      <c r="R199" t="inlineStr">
+        <is>
+          <t>OpenAlex API works/doi:10.24294/jipd9118; Abzal Omirbay L.N. Gumilyov Eurasian National University; Abzal Omirbay ORCID; сайт enu.kz преподаватели; Abzal Omirbay ResearchGate</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>moustafa_h</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Hanaa M. Moustafa</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Hanaa M. Moustafa</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>0009-0000-1837-4086</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Nursing Administration Department, Faculty of Nursing, Alexandria University, Egypt</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>Р4</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>Исследователь в области администрирования сестринского дела. Следов публичности в деловой среде не найдено — статья академическая, медицинская.</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>0009-0000-1837-4086</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI статьи 10.1186/s12912-024-02581-w; запись orcid.org недоступна</t>
+        </is>
+      </c>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>ждёт описания</t>
+        </is>
+      </c>
+      <c r="P200" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_06_effect_of_negotiation_skills_training_program_on_head_n</t>
+        </is>
+      </c>
+      <c r="R200" t="inlineStr">
+        <is>
+          <t>OpenAlex API по DOI; профиль Alexandria University; страница автора на сайте факультета</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>hassan_rm</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Rabab M. Hassan</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Rabab M. Hassan|Рабаб М. Хассан</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>0000-0001-7238-0034</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Department of Nursing Administration, Faculty of Nursing, Helwan University</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>Преподаватель кафедры сестринского администрирования факультета сестринского дела университета Хелуан, Каир. Исследует вопросы управления сестринским персоналом, программы обучения навыкам переговоров и разрешения конфликтов для руководителей среднего звена в медицинских организациях.</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>Исследователь в области сестринского администрирования с публикациями в рецензируемых журналах. Позиция в университете проверяема. Следов публичности в деловой среде или корпоративном обучении не найдено.</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>0000-0001-7238-0034</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI статьи 10.1186/s12912-024-02581-w; запись orcid.org недоступна</t>
+        </is>
+      </c>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P201" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_06_effect_of_negotiation_skills_training_program_on_head_n</t>
+        </is>
+      </c>
+      <c r="R201" t="inlineStr">
+        <is>
+          <t>openalex api doi:10.1186/s12912-024-02581-w; страница статьи bmcnursing; rabab hassan helwan university nursing</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>shakirov_s</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Symbat Shakirov</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Symbat Shakirov|Шакиров Символат Болтаевич|Shakirov Symbat Boltaevich</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>https://enu.kz/en/sotrudnik/shakirov-symbat-boltaevich/</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>страница_у_работодателя</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Professor, Head of the Department of Psychology and Pedagogy, L.N. Gumilyov Eurasian National University</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>Профессор, заведующий кафедрой психологии и педагогики Евразийского национального университета имени Л.Н. Гумилёва (Астана, Казахстан). PhD, область исследований: педагогическая психология, конфликтология в организациях, образовательные стратегии.</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>Позиция проверяема по странице работодателя. Следов в деловой среде не найдено: нет книг в деловых сериях, публикаций в HBR/Forbes/РБК/Ведомостях, спикерства на крупных корпоративных конференциях. Для корпоративной аудитории имя требует представления.</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>https://enu.kz/en/sotrudnik/shakirov-symbat-boltaevich/</t>
+        </is>
+      </c>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P202" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_05_Integration_Educational_Strategies</t>
+        </is>
+      </c>
+      <c r="R202" t="inlineStr">
+        <is>
+          <t>api.openalex.org/works/doi:10.24294/jipd9118; страница статьи https://doi.org/10.24294/jipd9118; site:enu.kz Symbat Shakirov; Shakirov Symbat Boltaevich Gumilyov University</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>badran_f</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Fawzia M. Badran</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Fawzia M. Badran|Фавзия М. Бадран</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>0000-0001-9694-9529</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Nursing Administration Department, Faculty of Nursing, Alexandria University</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>Преподаватель кафедры сестринского администрирования факультета сестринского дела Александрийского университета, Египет. Исследования в области управления конфликтами и переговорных навыков в сестринском менеджменте.</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>Академическая позиция в университете проверяема. Публикации в профильных научных журналах. Следов присутствия в деловой среде или корпоративном обучении не найдено.</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>0000-0001-9694-9529</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI статьи; запись orcid.org недоступна</t>
+        </is>
+      </c>
+      <c r="N203" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P203" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_06_effect_of_negotiation_skills_training_program_on_head_n</t>
+        </is>
+      </c>
+      <c r="R203" t="inlineStr">
+        <is>
+          <t>openalex api works by doi; fawzia badran alexandria university; fawzia badran nursing administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>mustafina_t</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Tolganay Mustafina</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Tolganay Mustafina|Толганай Мустафина</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>https://enu.kz/ru/sotrudnik/mustafina-tolganaj-anvarbekovna/</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>страница_у_работодателя</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>старший преподаватель, L.N. Gumilyov Eurasian National University</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>Старший преподаватель кафедры педагогики и психологии Евразийского национального университета имени Л.Н. Гумилёва (Астана, Казахстан). Исследует образовательные стратегии, конфликт-менеджмент в образовании, интеграцию цифровых технологий в педагогический процесс.</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>Р4</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>Преподаватель казахстанского университета, публикуется в академических журналах. Следов в русскоязычной или англоязычной деловой среде, корпоративных конференциях или бизнес-медиа не найдено.</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>https://enu.kz/ru/sotrudnik/mustafina-tolganaj-anvarbekovna/</t>
+        </is>
+      </c>
+      <c r="N204" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P204" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_05_Integration_Educational_Strategies</t>
+        </is>
+      </c>
+      <c r="R204" t="inlineStr">
+        <is>
+          <t>Tolganay Mustafina Gumilyov University; Mustafina педагогика психология ЕНУ; api.openalex.org/works/doi:10.24294/jipd9118; enu.kz staff Mustafina</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>baturin_v</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Vladimir Baturin</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Vladimir Baturin|Владимир Батурин</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>https://buketov.edu.kz/</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>страница_у_работодателя</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Buketov Karagandy University</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>Преподаватель Buketov Karagandy University (Караганда, Казахстан). Исследования в области образовательных стратегий и управления конфликтами в организациях.</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>Позиция в университете проверяема, публикация в международном журнале. Следов публичности в деловой среде или корпоративном обучении не найдено.</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>Страница автора на сайте Buketov Karagandy University https://buketov.edu.kz/</t>
+        </is>
+      </c>
+      <c r="N205" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P205" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_05_Integration_Educational_Strategies</t>
+        </is>
+      </c>
+      <c r="R205" t="inlineStr">
+        <is>
+          <t>Vladimir Baturin Buketov Karagandy University; api.openalex.org/works/doi:10.24294/jipd9118; Baturin Karagandy site:buketov.edu.kz; Vladimir Baturin ORCID</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>alsobay_m</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Mohammed Alsobay</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Mohammed Alsobay</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0002-8734-1803</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Microsoft Research</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>Исследователь в Microsoft Research. Работает в области human-AI interaction и computer-supported cooperative work (CSCW). Публикуется в области применения больших языковых моделей для групповой работы и принятия решений.</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>Исследователь в крупной корпоративной лаборатории, публикации в профильных научных конференциях (CHI, CSCW). Следов публичности в деловой среде или узнаваемости за пределами академического сообщества не найдено.</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>0000-0002-8734-1803</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>https://www.microsoft.com/en-us/research/people/moalsobay/</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI статьи 10.1145/3816907; запись orcid.org недоступна. Описание собрано со страницы автора Microsoft Research и профиля Google Scholar.</t>
+        </is>
+      </c>
+      <c r="N206" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P206" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_08_bringing_everyone_to_the_table_an_experimental_study_of</t>
+        </is>
+      </c>
+      <c r="R206" t="inlineStr">
+        <is>
+          <t>api.openalex.org/works/doi:10.1145/3816907; Mohammed Alsobay Microsoft Research; Mohammed Alsobay ORCID</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>rothschild_dm</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>David M. Rothschild</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>David M. Rothschild|Дэвид М. Ротшильд</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>0000-0002-5086-2805</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>Senior Principal Researcher, Microsoft Research</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>Senior Principal Researcher в Microsoft Research NYC, группа Computational Social Science. Исследует общественное мнение, прогнозирование и коллективное принятие решений. Публикуется в The New York Times, работает над применением машинного обучения к социальным данным.</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>Позиция в Microsoft Research проверяема, исследования цитируются в академической среде, публикации в The New York Times. Личной узнаваемости в русскоязычной корпоративной и деловой среде не установлено.</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>0000-0002-5086-2805</t>
+        </is>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>https://www.microsoft.com/en-us/research/people/dr/</t>
+        </is>
+      </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI 10.1145/3816907; запись orcid.org недоступна; профиль подтверждён страницей Microsoft Research</t>
+        </is>
+      </c>
+      <c r="N207" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P207" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_08_bringing_everyone_to_the_table_an_experimental_study_of</t>
+        </is>
+      </c>
+      <c r="R207" t="inlineStr">
+        <is>
+          <t>api.openalex.org/works/doi:10.1145/3816907; david rothschild microsoft research; страница статьи ACM Digital Library</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>hofman_j</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Jake M. Hofman</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Jake M. Hofman|Jake Hofman</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0002-9884-4160</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>Principal Researcher, Microsoft Research</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>Principal Researcher в Microsoft Research NYC. Исследует computational social science, предсказуемость человеческого поведения, машинное обучение в социальных системах. Публикуется в Science, PNAS, CHI, CSCW. Преподавал в Columbia University.</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>Р2</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>Публикации в топовых научных изданиях (Science, PNAS), выступления на конференциях (NeurIPS, WWW, CHI). Узнаваем в академической среде computational social science, следов в деловых медиа и русскоязычной корпоративной среде не найдено.</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>0000-0002-9884-4160</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>https://www.microsoft.com/en-us/research/people/jmh/</t>
+        </is>
+      </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI 10.1145/3816907; страница автора на сайте Microsoft Research подтверждает позицию и биографию</t>
+        </is>
+      </c>
+      <c r="N208" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P208" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_08_bringing_everyone_to_the_table_an_experimental_study_of</t>
+        </is>
+      </c>
+      <c r="R208" t="inlineStr">
+        <is>
+          <t>OpenAlex API: works/https://doi.org/10.1145/3816907; microsoft.com/research Jake Hofman; orcid.org/0000-0002-9884-4160 (недоступен напрямую, подтверждён через OpenAlex)</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>goldstein_dg</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Daniel G. Goldstein</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Daniel G. Goldstein|Daniel Goldstein</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>https://www.microsoft.com/en-us/research/people/dgg/</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>страница_у_работодателя</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Microsoft Research</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>Principal Researcher в Microsoft Research. Исследует применение поведенческой экономики и психологии принятия решений к дизайну технологий. Автор работ по персонализации рекомендаций, цифровому минимализму и применению AI в принятии групповых решений.</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>Р2</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>Публикуется в топовых научных конференциях (CHI, EC), статьи цитируются в академической среде поведенческой экономики и HCI. Работает в Microsoft Research — известной исследовательской лаборатории. Однако публичных следов в деловых медиа для широкой корпоративной аудитории не найдено — узнаваем в своей исследовательской нише.</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>0000-0002-6780-0089</t>
+        </is>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0002-6780-0089</t>
+        </is>
+      </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>Страница автора на сайте Microsoft Research https://www.microsoft.com/en-us/research/people/dgg/; ORCID 0000-0002-6780-0089 из метаданных OpenAlex по DOI 10.1145/3816907</t>
+        </is>
+      </c>
+      <c r="N209" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P209" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_08_bringing_everyone_to_the_table_an_experimental_study_of</t>
+        </is>
+      </c>
+      <c r="R209" t="inlineStr">
+        <is>
+          <t>openalex api works doi:10.1145/3816907; daniel goldstein microsoft research; daniel g goldstein behavioral economics</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>gimpel_h</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Henner Gimpel</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Henner Gimpel</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>0000-0003-1375-6059</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>профессор, заведующий кафедрой Digital Work and Human Resource Management, Университет Гогенгайма</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>Профессор цифровой работы и управления персоналом в Университете Гогенгайма (Hohenheim), заведующий кафедрой. Директор Центра интеллектуальных систем управления персоналом (CIHRS). Исследования фокусируются на цифровизации работы, ИИ в управлении персоналом, цифровом благополучии.</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>Профессор крупного немецкого университета, руководит исследовательским центром. Публикуется в академических журналах (Group Decision and Negotiation, др.). Следов в русскоязычной деловой среде или широкой узнаваемости среди практиков не найдено.</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>0000-0003-1375-6059</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>https://digital-work.uni-hohenheim.de/henner-gimpel</t>
+        </is>
+      </c>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI статьи; подтверждён страницей работодателя https://digital-work.uni-hohenheim.de/henner-gimpel</t>
+        </is>
+      </c>
+      <c r="N210" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P210" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_09_digital_facilitation_of_group_work_to_gain_predictable</t>
+        </is>
+      </c>
+      <c r="R210" t="inlineStr">
+        <is>
+          <t>api.openalex.org/works/https://doi.org/10.1007/s10726-023-09856-8; поиск 'Henner Gimpel University Hohenheim'; проверка страницы работодателя</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>wohl_m</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Moritz Wöhl</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Moritz Wöhl|Мориц Вёль</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>0000-0002-4994-1938</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>Научный сотрудник Information Management in Mechanical Engineering (IMA), факультет машиностроения RWTH Aachen University. Исследования сосредоточены на цифровой фасилитации групповой работы и управлении проектами.</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>Позиция в RWTH Aachen проверяема, публикации в академических журналах (Group Decision and Negotiation, Springer). Следов присутствия в деловой среде не найдено: нет публикаций в деловых медиа, книг, выступлений на корпоративных конференциях.</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>0000-0002-4994-1938</t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>https://www.ima.rwth-aachen.de/cms/IMA/Das-Institut/Mitarbeiter/~sezfi/Moritz-Woehl/</t>
+        </is>
+      </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI 10.1007/s10726-023-09856-8; описание со страницы автора на сайте RWTH Aachen University</t>
+        </is>
+      </c>
+      <c r="N211" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P211" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_09_digital_facilitation_of_group_work_to_gain_predictable</t>
+        </is>
+      </c>
+      <c r="R211" t="inlineStr">
+        <is>
+          <t>openalex api works doi; moritz wöhl rwth aachen; moritz wöhl digital facilitation; moritz wöhl hbr forbes; moritz wöhl conference speaker</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>graf-drasch_v</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Valerie Graf-Drasch</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Valerie Graf-Drasch</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>0000-0002-4734-7657</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>Исследователь в области информационных систем, University of Bayreuth. Работает над темами цифровой фасилитации, краудсорсинга и блокчейн-технологий в бизнес-процессах.</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>Исследователь с проверяемой позицией в университете, публикации в академических журналах (Group Decision and Negotiation, Electronic Markets). Публичных следов в русскоязычной или англоязычной деловой среде не найдено.</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>0000-0002-4734-7657</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>https://www.fim.uni-bayreuth.de/de/team/index.php?id=1201</t>
+        </is>
+      </c>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI статьи https://api.openalex.org/works/https://doi.org/10.1007/s10726-023-09856-8; профиль подтверждён страницей University of Bayreuth</t>
+        </is>
+      </c>
+      <c r="N212" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P212" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_09_digital_facilitation_of_group_work_to_gain_predictable</t>
+        </is>
+      </c>
+      <c r="R212" t="inlineStr">
+        <is>
+          <t>openalex api doi:10.1007/s10726-023-09856-8; valerie graf-drasch orcid; valerie graf-drasch university bayreuth</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>suharnomo</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Suharnomo</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Suharnomo</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?user=8cKHx8YAAAAJ</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>профиль_платформы</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>Профессор факультета экономики и бизнеса Университета Диponегоро (Индонезия), специализируется на управлении человеческими ресурсами и организационном поведении. Публикуется в журналах по менеджменту.</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>Профессор индонезийского университета, публикации в академических журналах по менеджменту. Позиция проверяема, следов в русскоязычной деловой среде не найдено.</t>
+        </is>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>https://sinta.kemdikbud.go.id/authors/profile/6004043</t>
+        </is>
+      </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>Google Scholar profile https://scholar.google.com/citations?user=8cKHx8YAAAAJ, SINTA (Science and Technology Index Indonesia) profile https://sinta.kemdikbud.go.id/authors/profile/6004043</t>
+        </is>
+      </c>
+      <c r="N213" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P213" t="inlineStr">
+        <is>
+          <t>Фокус на главном, долгосрочное планирование_02_Gaps_Empowering_Leadership</t>
+        </is>
+      </c>
+      <c r="R213" t="inlineStr">
+        <is>
+          <t>Suharnomo UMSurabaya; Suharnomo Diponegoro University; Suharnomo empowering leadership; Suharnomo ORCID</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>djastuti_i</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Indi Djastuti</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Indi Djastuti|И. Джастути</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>0000-0002-8494-0124</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>Lecturer, Department of Management, Universitas Muhammadiyah Surabaya</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>Преподаватель кафедры менеджмента факультета экономики и бизнеса Университета Мухаммадия Сурабая (Индонезия). Исследует организационное поведение, лидерство и управление персоналом, публикуется в международных журналах по менеджменту.</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>Р4</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>Исследователь регионального университета в Индонезии. Публикации в академических журналах, следов присутствия в русскоязычной или международной деловой среде не обнаружено. Имя не узнаваемо для корпоративной аудитории.</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>0000-0002-8494-0124</t>
+        </is>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>https://www.scopus.com/authid/detail.uri?authorId=57211495349</t>
+        </is>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>ORCID указан в метаданных публикаций на Scopus; запись orcid.org недоступна</t>
+        </is>
+      </c>
+      <c r="N214" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P214" t="inlineStr">
+        <is>
+          <t>Фокус на главном, долгосрочное планирование_02_Gaps_Empowering_Leadership, Фокус на главном, долгосрочное планирование_02_Gaps_Empowering_Leadership, Фокус на главном, долгосрочное планирование_02_Gaps_Empowering_Leadership</t>
+        </is>
+      </c>
+      <c r="R214" t="inlineStr">
+        <is>
+          <t>Indi Djastuti UMSurabaya; Indi Djastuti ORCID; Indi Djastuti empowering leadership; Indi Djastuti Universitas Muhammadiyah Surabaya</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>zierock_b</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Benjamin Zierock</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Benjamin Zierock</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>https://www.srh-heidelberg.de/en/university/about-us/organisation/people/benjamin-zierock/</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>страница_у_работодателя</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>SRH University Heidelberg</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>Профессор School of Applied Psychology в SRH University Heidelberg. Исследовательские интересы: цифровизация, организационное обучение, управление изменениями, OKR-методология. Публикуется по темам инноваций и agile-управления проектами.</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>Профессор немецкого университета, публикации в академических изданиях по OKR и управлению проектами. Деловых медиа, переводов книг, выступлений на корпоративных конференциях или собственной аудитории среди практиков не найдено.</t>
+        </is>
+      </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>https://www.srh-heidelberg.de/en/university/about-us/organisation/people/benjamin-zierock/</t>
+        </is>
+      </c>
+      <c r="N215" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P215" t="inlineStr">
+        <is>
+          <t>Фокус на главном, долгосрочное планирование_03_team_centric_innovation_the_role_of_objectives_and_key, Фокус на главном, долгосрочное планирование_03_team_centric_innovation_the_role_of_objectives_and_key</t>
+        </is>
+      </c>
+      <c r="R215" t="inlineStr">
+        <is>
+          <t>OpenAlex API по DOI 10.54941/ahfe1004717; поиск 'Benjamin Zierock SRH University Heidelberg'; сайт srh-heidelberg.de</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>blatz_m</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Matthias Blatz</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Matthias Blatz|Маттиас Блатц</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>https://heidelberg-it.management/team</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>страница_у_работодателя</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>консультант Heidelberg IT Management</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>Консультант Heidelberg IT Management GmbH &amp; Co. KG. Специализируется на цифровой трансформации, управлении проектами и внедрении agile-методологий в организациях.</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>Публикация в материалах конференции AHFE, работа в консалтинге. Публичных следов в деловых медиа, книг, выступлений на крупных конференциях не найдено.</t>
+        </is>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>https://heidelberg-it.management/team — профиль на сайте работодателя</t>
+        </is>
+      </c>
+      <c r="N216" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P216" t="inlineStr">
+        <is>
+          <t>Фокус на главном, долгосрочное планирование_03_team_centric_innovation_the_role_of_objectives_and_key, Фокус на главном, долгосрочное планирование_03_team_centric_innovation_the_role_of_objectives_and_key</t>
+        </is>
+      </c>
+      <c r="R216" t="inlineStr">
+        <is>
+          <t>openalex.org/works/doi:10.54941/ahfe1004717; heidelberg-it.management matthias blatz; matthias blatz orcid; matthias blatz linkedin</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>karcher_k</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Kris Karcher</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Kris Karcher</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>0000-0002-4863-3074</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>orcid</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>Applied AI Corporation Limited</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>Р4</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>Автор статей в академических сборниках по управлению проектами. Следов публичности в деловой среде (книги, колонки, конференции, кейсы) не найдено.</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>0000-0002-4863-3074</t>
+        </is>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>ORCID из метаданных OpenAlex по DOI 10.54941/ahfe1004717; запись orcid.org недоступна</t>
+        </is>
+      </c>
+      <c r="N217" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>ждёт описания</t>
+        </is>
+      </c>
+      <c r="P217" t="inlineStr">
+        <is>
+          <t>Фокус на главном, долгосрочное планирование_03_team_centric_innovation_the_role_of_objectives_and_key, Фокус на главном, долгосрочное планирование_03_team_centric_innovation_the_role_of_objectives_and_key</t>
+        </is>
+      </c>
+      <c r="R217" t="inlineStr">
+        <is>
+          <t>openalex works doi:10.54941/ahfe1004717; Kris Karcher Applied AI Corporation; Kris Karcher OKR project management; appliedai.co.uk team</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>lahmer_s</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Stefanie Lahmer</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Stefanie Lahmer</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>https://www.modul.ac.at/staff/stefanie-lahmer/</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>страница_у_работодателя</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>человек</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>Научный сотрудник MODUL University Vienna, специализируется на групповой динамике и цифровой фасилитации. Автор исследований в области управления конфликтами и организационного поведения.</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>Р3</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>Научный сотрудник университета, публикации в специализированных академических журналах. Позиция проверяема, публичных следов в русскоязычной или широкой деловой среде не найдено.</t>
+        </is>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>0000-0002-6219-394X</t>
+        </is>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>ORCID: 0000-0002-6219-394X из метаданных OpenAlex по DOI статьи</t>
+        </is>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>https://www.modul.ac.at/staff/stefanie-lahmer/</t>
+        </is>
+      </c>
+      <c r="N218" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>подтверждён</t>
+        </is>
+      </c>
+      <c r="P218" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_09_digital_facilitation_of_group_work_to_gain_predictable</t>
+        </is>
+      </c>
+      <c r="R218" t="inlineStr">
+        <is>
+          <t>OpenAlex API по DOI 10.1007/s10726-023-09856-8; страница статьи у издателя Springer; MODUL University Vienna staff page; Stefanie Lahmer MODUL University</t>
         </is>
       </c>
     </row>

</xml_diff>